<commit_message>
Add WorkflowType field distinguishing Legacy vs WFEngine automation systems
- parser: derive workflowType from export format — Legacy (embedded
  WorkflowConfigs in workspace export) or WFEngine (individual Triggers/Steps)
- build_inventory: WorkflowType column in Workflows sheet, amber/teal
  cell fill; TriggerGUID replaces the old Staging_GUID/Prod_GUID pair
- build_global: WorkflowType column in AllWorkflows sheet
- Both explorers: amber nodes for Legacy, red for WFEngine; [Legacy]/
  [WFEngine] label tag on each workflow node; legend updated
- CLAUDE.md: document what WorkflowType means and how it is derived

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$E$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$I$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'FormNameCollisions'!$A$3:$D$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DuplicateFlows'!$A$3:$D$7</definedName>
   </definedNames>
@@ -1936,17 +1936,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1974,25 +1975,30 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
+          <t>WorkflowType</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>TriggerForm</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>TriggerAction</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>TargetForms</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Writes</t>
         </is>
@@ -2016,25 +2022,30 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
+          <t>Legacy (embedded WorkflowConfigs) or WFEngine (Triggers/Steps)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
           <t>Active/Disabled</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Form that fires it</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Create/Update/Delete</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Forms it writes</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Field writes</t>
         </is>
@@ -2058,21 +2069,26 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>200 - Account</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr"/>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="9" t="inlineStr"/>
+      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2094,21 +2110,26 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>200 - Account</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2130,21 +2151,26 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2166,21 +2192,26 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2202,21 +2233,26 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="9" t="n">
+      <c r="H9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2238,17 +2274,22 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="n">
+      <c r="H10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2270,21 +2311,26 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr"/>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2306,21 +2352,26 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2342,21 +2393,26 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>255 - BE Installation Form</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr"/>
-      <c r="H13" s="9" t="n">
+      <c r="H13" s="9" t="inlineStr"/>
+      <c r="I13" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2378,21 +2434,26 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>255 - BE Installation Form</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2414,21 +2475,26 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>255 - BE Installation Form</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr"/>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2450,17 +2516,22 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>255 - BE Installation Form</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr"/>
       <c r="G16" s="9" t="inlineStr"/>
-      <c r="H16" s="9" t="n">
+      <c r="H16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2482,21 +2553,26 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>255 - BE Installation Form</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr"/>
-      <c r="H17" s="9" t="n">
+      <c r="H17" s="9" t="inlineStr"/>
+      <c r="I17" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2518,21 +2594,26 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr"/>
-      <c r="H18" s="9" t="n">
+      <c r="H18" s="9" t="inlineStr"/>
+      <c r="I18" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2554,21 +2635,26 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr"/>
-      <c r="H19" s="9" t="n">
+      <c r="H19" s="9" t="inlineStr"/>
+      <c r="I19" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2590,21 +2676,26 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr"/>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="9" t="inlineStr"/>
+      <c r="I20" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2626,21 +2717,26 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr"/>
-      <c r="H21" s="9" t="n">
+      <c r="H21" s="9" t="inlineStr"/>
+      <c r="I21" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2662,21 +2758,26 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
           <t>Disabled</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr"/>
-      <c r="H22" s="9" t="n">
+      <c r="H22" s="9" t="inlineStr"/>
+      <c r="I22" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2698,21 +2799,26 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr"/>
-      <c r="H23" s="9" t="n">
+      <c r="H23" s="9" t="inlineStr"/>
+      <c r="I23" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2734,21 +2840,26 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr"/>
-      <c r="H24" s="9" t="n">
+      <c r="H24" s="9" t="inlineStr"/>
+      <c r="I24" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2770,21 +2881,26 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr"/>
-      <c r="H25" s="9" t="n">
+      <c r="H25" s="9" t="inlineStr"/>
+      <c r="I25" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2806,21 +2922,26 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr"/>
-      <c r="H26" s="9" t="n">
+      <c r="H26" s="9" t="inlineStr"/>
+      <c r="I26" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2842,30 +2963,35 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
+          <t>WFEngine</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>300 - Account Management</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>395 - Inspection Work Order</t>
         </is>
       </c>
-      <c r="H27" s="9" t="n">
+      <c r="I27" s="9" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H27"/>
+  <autoFilter ref="A3:I27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>